<commit_message>
add : update Import create, update Employee and exportEmployee
</commit_message>
<xml_diff>
--- a/aspnet-core/src/HRMv2.Web.Host/wwwroot/template/Update-Employees.xlsx
+++ b/aspnet-core/src/HRMv2.Web.Host/wwwroot/template/Update-Employees.xlsx
@@ -1,40 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tool\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\quan.daominh\Documents\HRMv1\ncc-erp-hrm-v2\aspnet-core\src\HRMv2.Web.Host\wwwroot\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F76A864-41E2-41ED-89BD-4431B8DAC3D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{991EC3D6-06E7-4F38-AD24-FEFB9BE04CDE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8988" xr2:uid="{15B0A3F3-DF1A-4DF6-A8BB-08B5516BAA62}"/>
+    <workbookView xWindow="765" yWindow="765" windowWidth="17280" windowHeight="8985" xr2:uid="{15B0A3F3-DF1A-4DF6-A8BB-08B5516BAA62}"/>
   </bookViews>
   <sheets>
     <sheet name="Employee" sheetId="1" r:id="rId1"/>
     <sheet name="Metadata" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <externalReferences>
+    <externalReference r:id="rId3"/>
+  </externalReferences>
+  <calcPr calcId="179021"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="25">
   <si>
     <t>Email*</t>
   </si>
@@ -106,6 +101,9 @@
   </si>
   <si>
     <t>StartWorkingDate</t>
+  </si>
+  <si>
+    <t>MezonUserId</t>
   </si>
 </sst>
 </file>
@@ -170,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -181,6 +179,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -198,10 +199,25 @@
 </styleSheet>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Employee"/>
+      <sheetName val="Metadata"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -239,7 +255,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -345,7 +361,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -487,7 +503,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -495,24 +511,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8A9D128-3347-4177-A648-6A7D7A6B6DDD}">
-  <dimension ref="A1:O1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:P2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.6640625" customWidth="1"/>
-    <col min="2" max="3" width="23.88671875" style="2" customWidth="1"/>
-    <col min="4" max="6" width="25.88671875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="29.33203125" customWidth="1"/>
+    <col min="1" max="1" width="30.7109375" customWidth="1"/>
+    <col min="2" max="3" width="23.85546875" style="2" customWidth="1"/>
+    <col min="4" max="6" width="25.85546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="29.28515625" customWidth="1"/>
     <col min="8" max="8" width="29" customWidth="1"/>
-    <col min="9" max="9" width="27.5546875" customWidth="1"/>
+    <col min="9" max="9" width="27.5703125" customWidth="1"/>
     <col min="10" max="10" width="19" customWidth="1"/>
-    <col min="11" max="11" width="15.5546875" customWidth="1"/>
-    <col min="12" max="12" width="44.6640625" customWidth="1"/>
-    <col min="13" max="13" width="36.109375" customWidth="1"/>
-    <col min="14" max="14" width="17.44140625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5703125" customWidth="1"/>
+    <col min="12" max="12" width="44.7109375" customWidth="1"/>
+    <col min="13" max="13" width="36.140625" customWidth="1"/>
+    <col min="14" max="14" width="17.42578125" style="1" customWidth="1"/>
     <col min="15" max="15" width="33" customWidth="1"/>
+    <col min="16" max="16" width="15.28515625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="4" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" s="4" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -558,6 +575,18 @@
       <c r="O1" s="8" t="s">
         <v>11</v>
       </c>
+      <c r="P1" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="P2" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -565,17 +594,17 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B1BF61F6-C7E6-4645-A02E-E2D4612245E9}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3D4ECA59-B237-46F1-A5F4-7C039437D80C}">
           <x14:formula1>
-            <xm:f>Metadata!$B$2:$B$4</xm:f>
+            <xm:f>'[Update-Employees-1.xlsx]Metadata'!#REF!</xm:f>
+          </x14:formula1>
+          <xm:sqref>G2</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8B52B05A-11B1-4C66-B215-9D3E935E9697}">
+          <x14:formula1>
+            <xm:f>'[Update-Employees-1.xlsx]Metadata'!#REF!</xm:f>
           </x14:formula1>
           <xm:sqref>J2</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{CA7250F3-3039-4454-95D8-EAF0080C9882}">
-          <x14:formula1>
-            <xm:f>Metadata!$A$2:$A$25</xm:f>
-          </x14:formula1>
-          <xm:sqref>G2</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -586,13 +615,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{205B96B4-0DD7-48F9-84EC-9A8587ADC8D5}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>3</v>
       </c>
@@ -600,7 +629,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>12</v>
       </c>
@@ -608,7 +637,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -616,7 +645,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -624,7 +653,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -632,7 +661,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>

</xml_diff>